<commit_message>
Add rl (reinsurance loss/ceded) as a well-known perspective_code value
Oasis produces both the net RI loss (ri — the cedant's retained loss after
reinsurance recoveries) and the ceded RI loss (the amount recovered from
reinsurers) as separate perspectives; only ri was documented. Adds rl
alongside gul/il/ri everywhere the well-known perspective_code values are
listed: the metadata schema, its human-readable doc, the Perspectives CSV
note, and the matching note in ORD_Data_Spec.xlsx.

perspective_code remains a free string (not an enum) in both the JSON
schema and the relational model, so this is a documentation-only change.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/ORD_Data_Spec.xlsx
+++ b/Docs/ORD_Data_Spec.xlsx
@@ -1248,7 +1248,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H59"/>
+  <dimension ref="B1:H59"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="2.6640625" customWidth="1" style="61" min="1" max="1"/>
@@ -10477,8 +10477,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12"/>
     <row r="13">
       <c r="B13" s="89" t="n"/>
     </row>
@@ -10984,7 +10982,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="B1:I19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="2.6640625" customWidth="1" style="61" min="1" max="1"/>
@@ -11003,7 +11001,7 @@
     <row r="3">
       <c r="B3" t="inlineStr">
         <is>
-          <t>ORD v2 note: perspective_code is a free string, not a locked enum. Well-known Oasis/OED values are gul, il, ri. The list below is illustrative of possible perspectives, not exhaustive or fixed.</t>
+          <t>ORD v2 note: perspective_code is a free string, not a locked enum. Well-known Oasis/OED values are gul, il, ri (reinsurance net, i.e. cedant's retained loss), and rl (reinsurance loss, i.e. ceded amount recovered from reinsurers). The list below is illustrative of possible perspectives, not exhaustive or fixed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove C_PARA EPMethod and c_para_distribution_type from ORD v2
C_PARA (convolution with parametric uncertainty) and the associated
results-metadata field c_para_distribution_type came from a pre-meeting
discussion document. The working group decided at the 2 Sep 2026 call
(reconfirmed afterwards by email) that they are not needed: Verisk does
not use severity distributions for its uncertainty EP curves, so there
is no parametric-convolution EP variant to represent.

The ORD v2 EPMethod codes are therefore A_MEAN, S_FULL, S_PSMN, S_MEAN
and C_MEAN.

Removed from:
- Create_ORDB_v2_0.sql: EPMethod seed row, Settings column, changelog
- results_metadata_schema_v2.json/.md: ep_methods description and the
  c_para_distribution_type property
- ORD_Definitions.md, ORD_List_of_Fields.csv, ORD_Table_Examples.csv
- Docs/ORD_Data_Spec.xlsx

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/ORD_Data_Spec.xlsx
+++ b/Docs/ORD_Data_Spec.xlsx
@@ -2477,7 +2477,7 @@
       <c r="BP12" s="66" t="n"/>
       <c r="CI12" t="inlineStr">
         <is>
-          <t>EPMethod: A_MEAN, S_FULL, S_PSMN, S_MEAN, C_MEAN, C_PARA</t>
+          <t>EPMethod: A_MEAN, S_FULL, S_PSMN, S_MEAN, C_MEAN</t>
         </is>
       </c>
       <c r="CO12" t="inlineStr">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="G124" s="38" t="inlineStr">
         <is>
-          <t>String code for EP calculation method (ORD v2): A_MEAN, S_FULL, S_PSMN, S_MEAN, C_MEAN, C_PARA. Prefix indicates LossMethod (A_=MEAN, S_=STOC, C_=CONV).</t>
+          <t>String code for EP calculation method (ORD v2): A_MEAN, S_FULL, S_PSMN, S_MEAN, C_MEAN. Prefix indicates LossMethod (A_=MEAN, S_=STOC, C_=CONV).</t>
         </is>
       </c>
       <c r="H124" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Add GELT to the CSVs/xlsx and align all lookup tables on ShortName
- Add GELT to ORD_Tables.csv, ORD_List_of_Fields.csv (14 field rows,
  including GroupMethod/GroupEventSetId, with the RSAM restriction noted)
  and ORD_Data_Types.csv, and mirror these in ORD_Data_Spec.xlsx.
  ORD_Table_Examples.csv has no grouped-table examples yet, so GELT isn't
  added there either.
- GroupMethod: drop LegacyInt. GroupMethod is new in v2 so it has no v1
  integer to trace. Drop the Int column from its table in ORD_Definitions.md.
- LossMethod: Description -> ShortName, so every lookup table uses
  ShortName.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/ORD_Data_Spec.xlsx
+++ b/Docs/ORD_Data_Spec.xlsx
@@ -16,7 +16,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perspectives" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tables'!$B$4:$H$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tables'!$B$4:$H$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'ListOfFields'!$B$7:$I$124</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -1248,7 +1248,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:H59"/>
+  <dimension ref="A1:H60"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="2.6640625" customWidth="1" style="61" min="1" max="1"/>
@@ -1268,6 +1268,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="16" customHeight="1" s="61">
       <c r="B3" s="13" t="n"/>
     </row>
@@ -1710,33 +1711,36 @@
       </c>
     </row>
     <row r="17" ht="32" customHeight="1" s="61">
-      <c r="B17" s="32" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Results</t>
         </is>
       </c>
-      <c r="C17" s="33" t="inlineStr">
-        <is>
-          <t>Error Log</t>
-        </is>
-      </c>
-      <c r="D17" s="54" t="inlineStr">
-        <is>
-          <t>ELOG</t>
-        </is>
-      </c>
-      <c r="E17" s="33" t="inlineStr">
-        <is>
-          <t>Contains error codes for locations that were failed to be processed by the model</t>
-        </is>
-      </c>
-      <c r="F17" s="34" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G17" s="34" t="n"/>
-      <c r="H17" s="33" t="n"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Group Event Loss Table</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>GELT</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Grouped event losses combining compatible analyses (ORD v2); uses GroupMethod (MEAN or RSSD only, not valid for RSAM) and requires GroupEventSetId</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>GroupMethod column (new in ORD v2)</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="32" customHeight="1" s="61">
       <c r="B18" s="32" t="inlineStr">
@@ -1746,22 +1750,22 @@
       </c>
       <c r="C18" s="33" t="inlineStr">
         <is>
-          <t>Aggregate summaries of exposure within model domain</t>
+          <t>Error Log</t>
         </is>
       </c>
       <c r="D18" s="54" t="inlineStr">
         <is>
-          <t>DOMEXP</t>
+          <t>ELOG</t>
         </is>
       </c>
       <c r="E18" s="33" t="inlineStr">
         <is>
-          <t>Model specific so needs to be in the Results area</t>
+          <t>Contains error codes for locations that were failed to be processed by the model</t>
         </is>
       </c>
       <c r="F18" s="34" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G18" s="34" t="n"/>
@@ -1775,12 +1779,12 @@
       </c>
       <c r="C19" s="33" t="inlineStr">
         <is>
-          <t>Aggregate summaries of rejected exposure by reason rejected</t>
+          <t>Aggregate summaries of exposure within model domain</t>
         </is>
       </c>
       <c r="D19" s="54" t="inlineStr">
         <is>
-          <t>REJEXP</t>
+          <t>DOMEXP</t>
         </is>
       </c>
       <c r="E19" s="33" t="inlineStr">
@@ -1797,49 +1801,49 @@
       <c r="H19" s="33" t="n"/>
     </row>
     <row r="20" ht="16" customHeight="1" s="61">
-      <c r="B20" s="35" t="inlineStr">
-        <is>
-          <t>Analysis</t>
-        </is>
-      </c>
-      <c r="C20" s="75" t="inlineStr">
-        <is>
-          <t>Analysis MetaData json blob - see example</t>
-        </is>
-      </c>
-      <c r="D20" s="37" t="n"/>
-      <c r="E20" s="38" t="inlineStr">
-        <is>
-          <t>File that includes metadata for each analysis. It ties everything together and enables full audit trail.</t>
-        </is>
-      </c>
-      <c r="F20" s="41" t="inlineStr">
-        <is>
-          <t>partly</t>
-        </is>
-      </c>
-      <c r="G20" s="41" t="inlineStr">
-        <is>
-          <t>analysis_settings</t>
-        </is>
-      </c>
-      <c r="H20" s="38" t="n"/>
+      <c r="B20" s="32" t="inlineStr">
+        <is>
+          <t>Results</t>
+        </is>
+      </c>
+      <c r="C20" s="33" t="inlineStr">
+        <is>
+          <t>Aggregate summaries of rejected exposure by reason rejected</t>
+        </is>
+      </c>
+      <c r="D20" s="54" t="inlineStr">
+        <is>
+          <t>REJEXP</t>
+        </is>
+      </c>
+      <c r="E20" s="33" t="inlineStr">
+        <is>
+          <t>Model specific so needs to be in the Results area</t>
+        </is>
+      </c>
+      <c r="F20" s="34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G20" s="34" t="n"/>
+      <c r="H20" s="33" t="n"/>
     </row>
     <row r="21" ht="16" customHeight="1" s="61">
       <c r="B21" s="35" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>Analysis</t>
         </is>
       </c>
       <c r="C21" s="75" t="inlineStr">
         <is>
-          <t>Model MetaData json blob - not done yet</t>
+          <t>Analysis MetaData json blob - see example</t>
         </is>
       </c>
       <c r="D21" s="37" t="n"/>
       <c r="E21" s="38" t="inlineStr">
         <is>
-          <t>A file that gives mandatory information about each model, including name, version number, frequency, severity and seasonality usage</t>
+          <t>File that includes metadata for each analysis. It ties everything together and enables full audit trail.</t>
         </is>
       </c>
       <c r="F21" s="41" t="inlineStr">
@@ -1847,7 +1851,11 @@
           <t>partly</t>
         </is>
       </c>
-      <c r="G21" s="41" t="n"/>
+      <c r="G21" s="41" t="inlineStr">
+        <is>
+          <t>analysis_settings</t>
+        </is>
+      </c>
       <c r="H21" s="38" t="n"/>
     </row>
     <row r="22" ht="16" customHeight="1" s="61">
@@ -1856,20 +1864,20 @@
           <t>Model</t>
         </is>
       </c>
-      <c r="C22" s="38" t="inlineStr">
-        <is>
-          <t>Event</t>
+      <c r="C22" s="75" t="inlineStr">
+        <is>
+          <t>Model MetaData json blob - not done yet</t>
         </is>
       </c>
       <c r="D22" s="37" t="n"/>
       <c r="E22" s="38" t="inlineStr">
         <is>
-          <t>Contains the full set of events with optional event descriptions and the event rate provided by the modeller as well as, optionally, an OriginalEventRate field</t>
+          <t>A file that gives mandatory information about each model, including name, version number, frequency, severity and seasonality usage</t>
         </is>
       </c>
       <c r="F22" s="41" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>partly</t>
         </is>
       </c>
       <c r="G22" s="41" t="n"/>
@@ -1883,13 +1891,13 @@
       </c>
       <c r="C23" s="38" t="inlineStr">
         <is>
-          <t>Occurrence</t>
+          <t>Event</t>
         </is>
       </c>
       <c r="D23" s="37" t="n"/>
       <c r="E23" s="38" t="inlineStr">
         <is>
-          <t>If we add an optional quantile column and then this can also serve as the RMS style PEQT</t>
+          <t>Contains the full set of events with optional event descriptions and the event rate provided by the modeller as well as, optionally, an OriginalEventRate field</t>
         </is>
       </c>
       <c r="F23" s="41" t="inlineStr">
@@ -1908,13 +1916,13 @@
       </c>
       <c r="C24" s="38" t="inlineStr">
         <is>
-          <t>Event Footprint</t>
+          <t>Occurrence</t>
         </is>
       </c>
       <c r="D24" s="37" t="n"/>
       <c r="E24" s="38" t="inlineStr">
         <is>
-          <t>Contains information about the footprint of each event</t>
+          <t>If we add an optional quantile column and then this can also serve as the RMS style PEQT</t>
         </is>
       </c>
       <c r="F24" s="41" t="inlineStr">
@@ -1933,13 +1941,13 @@
       </c>
       <c r="C25" s="38" t="inlineStr">
         <is>
-          <t>Vulnerability</t>
+          <t>Event Footprint</t>
         </is>
       </c>
       <c r="D25" s="37" t="n"/>
       <c r="E25" s="38" t="inlineStr">
         <is>
-          <t>Contains information about each vulnerability curve</t>
+          <t>Contains information about the footprint of each event</t>
         </is>
       </c>
       <c r="F25" s="41" t="inlineStr">
@@ -1958,13 +1966,13 @@
       </c>
       <c r="C26" s="38" t="inlineStr">
         <is>
-          <t>Period Weights</t>
+          <t>Vulnerability</t>
         </is>
       </c>
       <c r="D26" s="37" t="n"/>
       <c r="E26" s="38" t="inlineStr">
         <is>
-          <t>Or we could include PeriodWeight as an optional column in the Occurrence file</t>
+          <t>Contains information about each vulnerability curve</t>
         </is>
       </c>
       <c r="F26" s="41" t="inlineStr">
@@ -1976,29 +1984,29 @@
       <c r="H26" s="38" t="n"/>
     </row>
     <row r="27">
-      <c r="B27" s="32" t="inlineStr">
-        <is>
-          <t>Exposure</t>
-        </is>
-      </c>
-      <c r="C27" s="33" t="inlineStr">
-        <is>
-          <t>Input Exposure</t>
-        </is>
-      </c>
-      <c r="D27" s="54" t="n"/>
-      <c r="E27" s="33" t="inlineStr">
-        <is>
-          <t>Table for each input file: 2 or 4 for OED (with &amp; without RI),  different numbers of files for other vendors</t>
-        </is>
-      </c>
-      <c r="F27" s="34" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G27" s="34" t="n"/>
-      <c r="H27" s="33" t="n"/>
+      <c r="B27" s="35" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="C27" s="38" t="inlineStr">
+        <is>
+          <t>Period Weights</t>
+        </is>
+      </c>
+      <c r="D27" s="37" t="n"/>
+      <c r="E27" s="38" t="inlineStr">
+        <is>
+          <t>Or we could include PeriodWeight as an optional column in the Occurrence file</t>
+        </is>
+      </c>
+      <c r="F27" s="41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G27" s="41" t="n"/>
+      <c r="H27" s="38" t="n"/>
     </row>
     <row r="28">
       <c r="B28" s="32" t="inlineStr">
@@ -2008,13 +2016,13 @@
       </c>
       <c r="C28" s="33" t="inlineStr">
         <is>
-          <t>Aggregated Exposure</t>
+          <t>Input Exposure</t>
         </is>
       </c>
       <c r="D28" s="54" t="n"/>
       <c r="E28" s="33" t="inlineStr">
         <is>
-          <t>Aggregate summaries of input exposure</t>
+          <t>Table for each input file: 2 or 4 for OED (with &amp; without RI),  different numbers of files for other vendors</t>
         </is>
       </c>
       <c r="F28" s="34" t="inlineStr">
@@ -2026,32 +2034,51 @@
       <c r="H28" s="33" t="n"/>
     </row>
     <row r="29">
-      <c r="B29" s="35" t="inlineStr">
+      <c r="B29" s="32" t="inlineStr">
+        <is>
+          <t>Exposure</t>
+        </is>
+      </c>
+      <c r="C29" s="33" t="inlineStr">
+        <is>
+          <t>Aggregated Exposure</t>
+        </is>
+      </c>
+      <c r="D29" s="54" t="n"/>
+      <c r="E29" s="33" t="inlineStr">
+        <is>
+          <t>Aggregate summaries of input exposure</t>
+        </is>
+      </c>
+      <c r="F29" s="34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G29" s="34" t="n"/>
+      <c r="H29" s="33" t="n"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="35" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="C29" s="38" t="inlineStr">
+      <c r="C30" s="38" t="inlineStr">
         <is>
           <t>Shapefiles</t>
         </is>
       </c>
-      <c r="E29" s="38" t="inlineStr">
+      <c r="E30" s="38" t="inlineStr">
         <is>
           <t>The possibility of including shapefiles should be included</t>
         </is>
       </c>
-      <c r="F29" s="41" t="inlineStr">
+      <c r="F30" s="41" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G29" s="41" t="n"/>
-      <c r="H29" s="38" t="n"/>
-    </row>
-    <row r="30">
-      <c r="E30" s="38" t="n"/>
-      <c r="F30" s="38" t="n"/>
       <c r="G30" s="41" t="n"/>
       <c r="H30" s="38" t="n"/>
     </row>
@@ -2229,8 +2256,14 @@
       <c r="G59" s="41" t="n"/>
       <c r="H59" s="38" t="n"/>
     </row>
+    <row r="60">
+      <c r="E60" s="38" t="n"/>
+      <c r="F60" s="38" t="n"/>
+      <c r="G60" s="41" t="n"/>
+      <c r="H60" s="38" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="B4:H26"/>
+  <autoFilter ref="B4:H27"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
   <pageSetup orientation="portrait" paperSize="9" firstPageNumber="0" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -2342,19 +2375,15 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="B5" s="86" t="n"/>
     </row>
     <row r="6">
       <c r="B6" s="86" t="n"/>
     </row>
-    <row r="7"/>
-    <row r="8"/>
     <row r="9">
       <c r="CI9" s="86" t="n"/>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="B11" s="66" t="inlineStr">
         <is>
@@ -4960,15 +4989,6 @@
       </c>
       <c r="AQ43" s="58" t="n"/>
     </row>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
     <row r="53">
       <c r="B53" s="66" t="n"/>
     </row>
@@ -4984,7 +5004,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI19"/>
+  <dimension ref="A1:AL19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="13"/>
   <cols>
     <col width="21.1640625" customWidth="1" style="111" min="1" max="1"/>
@@ -5017,6 +5037,8 @@
     <col width="13" customWidth="1" style="61" min="34" max="34"/>
     <col width="13" customWidth="1" style="61" min="35" max="35"/>
     <col width="13" customWidth="1" style="61" min="36" max="36"/>
+    <col width="13" customWidth="1" style="61" min="37" max="37"/>
+    <col width="13" customWidth="1" style="61" min="38" max="38"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5080,6 +5102,11 @@
           <t>GEPT</t>
         </is>
       </c>
+      <c r="AK1" s="113" t="inlineStr">
+        <is>
+          <t>GELT</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="112" t="inlineStr">
@@ -5202,6 +5229,16 @@
           <t>Data Type</t>
         </is>
       </c>
+      <c r="AK2" s="112" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="AL2" s="112" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="111" t="inlineStr">
@@ -5324,6 +5361,16 @@
           <t>string</t>
         </is>
       </c>
+      <c r="AK3" s="111" t="inlineStr">
+        <is>
+          <t>GroupEventSetId</t>
+        </is>
+      </c>
+      <c r="AL3" s="111" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="111" t="inlineStr">
@@ -5446,6 +5493,16 @@
           <t>32-bit integer</t>
         </is>
       </c>
+      <c r="AK4" s="111" t="inlineStr">
+        <is>
+          <t>SummaryId</t>
+        </is>
+      </c>
+      <c r="AL4" s="111" t="inlineStr">
+        <is>
+          <t>32-bit integer</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="111" t="inlineStr">
@@ -5568,6 +5625,16 @@
           <t>string</t>
         </is>
       </c>
+      <c r="AK5" s="111" t="inlineStr">
+        <is>
+          <t>EventId</t>
+        </is>
+      </c>
+      <c r="AL5" s="111" t="inlineStr">
+        <is>
+          <t>32-bit integer</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="111" t="inlineStr">
@@ -5690,6 +5757,16 @@
           <t>float</t>
         </is>
       </c>
+      <c r="AK6" s="111" t="inlineStr">
+        <is>
+          <t>GroupMethod</t>
+        </is>
+      </c>
+      <c r="AL6" s="111" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="111" t="inlineStr">
@@ -5802,6 +5879,16 @@
           <t>float</t>
         </is>
       </c>
+      <c r="AK7" s="111" t="inlineStr">
+        <is>
+          <t>EventRate</t>
+        </is>
+      </c>
+      <c r="AL7" s="111" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="111" t="inlineStr">
@@ -5864,6 +5951,16 @@
           <t>float</t>
         </is>
       </c>
+      <c r="AK8" t="inlineStr">
+        <is>
+          <t>ChanceOfLoss</t>
+        </is>
+      </c>
+      <c r="AL8" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="111" t="inlineStr">
@@ -5916,6 +6013,16 @@
           <t>float</t>
         </is>
       </c>
+      <c r="AK9" t="inlineStr">
+        <is>
+          <t>MeanLoss</t>
+        </is>
+      </c>
+      <c r="AL9" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="111" t="inlineStr">
@@ -5958,6 +6065,16 @@
           <t>float</t>
         </is>
       </c>
+      <c r="AK10" t="inlineStr">
+        <is>
+          <t>SDLoss</t>
+        </is>
+      </c>
+      <c r="AL10" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="111" t="inlineStr">
@@ -6000,6 +6117,16 @@
           <t>float</t>
         </is>
       </c>
+      <c r="AK11" t="inlineStr">
+        <is>
+          <t>MaxLoss</t>
+        </is>
+      </c>
+      <c r="AL11" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="111" t="inlineStr">
@@ -6042,6 +6169,16 @@
           <t>float</t>
         </is>
       </c>
+      <c r="AK12" t="inlineStr">
+        <is>
+          <t>FootprintExposure</t>
+        </is>
+      </c>
+      <c r="AL12" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="111" t="inlineStr">
@@ -6084,6 +6221,16 @@
           <t>float</t>
         </is>
       </c>
+      <c r="AK13" t="inlineStr">
+        <is>
+          <t>MeanImpactedExposure</t>
+        </is>
+      </c>
+      <c r="AL13" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="111" t="inlineStr">
@@ -6106,6 +6253,16 @@
           <t>float</t>
         </is>
       </c>
+      <c r="AK14" t="inlineStr">
+        <is>
+          <t>MaxImpactedExposure</t>
+        </is>
+      </c>
+      <c r="AL14" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="111" t="inlineStr">
@@ -6118,6 +6275,16 @@
           <t>float</t>
         </is>
       </c>
+      <c r="AK15" t="inlineStr">
+        <is>
+          <t>SDLossCor</t>
+        </is>
+      </c>
+      <c r="AL15" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="111" t="inlineStr">
@@ -6130,6 +6297,16 @@
           <t>float</t>
         </is>
       </c>
+      <c r="AK16" t="inlineStr">
+        <is>
+          <t>SDLossInd</t>
+        </is>
+      </c>
+      <c r="AL16" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="111" t="inlineStr">
@@ -6168,13 +6345,14 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="13">
     <mergeCell ref="AB1:AC1"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="V1:W1"/>
     <mergeCell ref="S1:T1"/>
     <mergeCell ref="AH1:AI1"/>
+    <mergeCell ref="AK1:AL1"/>
     <mergeCell ref="J1:K1"/>
     <mergeCell ref="Y1:Z1"/>
     <mergeCell ref="P1:Q1"/>
@@ -6202,7 +6380,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I159"/>
+  <dimension ref="B1:I159"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="2.6640625" customWidth="1" style="61" min="1" max="1"/>
@@ -6298,7 +6476,7 @@
       </c>
       <c r="C8" s="76" t="inlineStr">
         <is>
-          <t>ALT,EPT,PSEPT,MELT,MPLT,SELT,SPLT,QELT,QPLT,GPLT,GALT,GEPT</t>
+          <t>ALT,EPT,PSEPT,MELT,MPLT,SELT,SPLT,QELT,QPLT,GPLT,GALT,GEPT,GELT</t>
         </is>
       </c>
       <c r="D8" s="76" t="inlineStr">
@@ -6368,7 +6546,7 @@
       </c>
       <c r="C10" s="76" t="inlineStr">
         <is>
-          <t>ALT,MELT,MPLT,GALT</t>
+          <t>ALT,MELT,MPLT,GALT,GELT</t>
         </is>
       </c>
       <c r="D10" s="76" t="inlineStr">
@@ -6401,7 +6579,7 @@
       </c>
       <c r="C11" s="76" t="inlineStr">
         <is>
-          <t>ALT,MELT,MPLT,GALT</t>
+          <t>ALT,MELT,MPLT,GALT,GELT</t>
         </is>
       </c>
       <c r="D11" s="76" t="inlineStr">
@@ -6467,7 +6645,7 @@
       </c>
       <c r="C13" s="76" t="inlineStr">
         <is>
-          <t>MELT,MPLT</t>
+          <t>MELT,MPLT,GELT</t>
         </is>
       </c>
       <c r="D13" s="76" t="inlineStr">
@@ -6673,7 +6851,7 @@
       </c>
       <c r="C19" s="76" t="inlineStr">
         <is>
-          <t>MELT,MPLT,SELT,SPLT,QELT,QPLT,GPLT</t>
+          <t>MELT,MPLT,SELT,SPLT,QELT,QPLT,GPLT,GELT</t>
         </is>
       </c>
       <c r="D19" s="76" t="inlineStr">
@@ -6906,7 +7084,7 @@
       </c>
       <c r="C26" s="71" t="inlineStr">
         <is>
-          <t>MELT</t>
+          <t>MELT,GELT</t>
         </is>
       </c>
       <c r="D26" s="76" t="inlineStr">
@@ -7054,7 +7232,7 @@
       </c>
       <c r="C30" s="71" t="inlineStr">
         <is>
-          <t>MELT,MPLT</t>
+          <t>MELT,MPLT,GELT</t>
         </is>
       </c>
       <c r="D30" s="76" t="inlineStr">
@@ -7088,7 +7266,7 @@
       </c>
       <c r="C31" s="71" t="inlineStr">
         <is>
-          <t>MELT,MPLT</t>
+          <t>MELT,MPLT,GELT</t>
         </is>
       </c>
       <c r="D31" s="76" t="inlineStr">
@@ -10193,7 +10371,7 @@
       </c>
       <c r="C118" s="76" t="inlineStr">
         <is>
-          <t>MELT, MPLT</t>
+          <t>MELT, MPLT, GELT</t>
         </is>
       </c>
       <c r="D118" s="76" t="inlineStr">
@@ -10230,7 +10408,7 @@
       </c>
       <c r="C119" s="76" t="inlineStr">
         <is>
-          <t>MELT, MPLT</t>
+          <t>MELT, MPLT, GELT</t>
         </is>
       </c>
       <c r="D119" s="76" t="inlineStr">
@@ -10267,7 +10445,7 @@
       </c>
       <c r="C120" s="71" t="inlineStr">
         <is>
-          <t>MELT,MPLT</t>
+          <t>MELT,MPLT,GELT</t>
         </is>
       </c>
       <c r="D120" s="76" t="inlineStr">
@@ -10300,7 +10478,7 @@
       </c>
       <c r="C121" s="71" t="inlineStr">
         <is>
-          <t>MELT,MPLT</t>
+          <t>MELT,MPLT,GELT</t>
         </is>
       </c>
       <c r="D121" s="76" t="inlineStr">
@@ -10546,7 +10724,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>GPLT,GALT,GEPT</t>
+          <t>GPLT,GALT,GEPT,GELT</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -10561,7 +10739,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>String code for grouped-analysis calculation method: MEAN, RSAM, RSSD. Used on grouped output tables in place of EPMethod (no EP variants needed); MEAN LossMethod is excluded as a GroupMethod.</t>
+          <t>String code for grouped-analysis calculation method: MEAN, RSAM, RSSD. Used on grouped output tables in place of EPMethod (no EP variants needed); MEAN LossMethod is excluded as a GroupMethod. GELT is valid for MEAN and RSSD only, not RSAM.</t>
         </is>
       </c>
       <c r="H128" s="38" t="inlineStr">
@@ -10583,7 +10761,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>GPLT,GALT,GEPT</t>
+          <t>GPLT,GALT,GEPT,GELT</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">

</xml_diff>